<commit_message>
Correct preload and accept loadstep diff in bolts config
</commit_message>
<xml_diff>
--- a/tests/bolts/res/Flange1.xlsx
+++ b/tests/bolts/res/Flange1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATA\laghida\Documents\GitLab\cassy\tests\bolts\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3F5DA06-146D-4401-9909-6A721E41DA7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DF3670D-C405-47F8-832A-B70F76F4E489}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="55">
   <si>
     <t>ID</t>
   </si>
@@ -96,9 +96,6 @@
     <t>SMHV</t>
   </si>
   <si>
-    <t>loads_3</t>
-  </si>
-  <si>
     <t>III</t>
   </si>
   <si>
@@ -117,9 +114,6 @@
     <t>SL2</t>
   </si>
   <si>
-    <t>loads_4</t>
-  </si>
-  <si>
     <t>IV</t>
   </si>
   <si>
@@ -138,9 +132,6 @@
     <t>Assembly</t>
   </si>
   <si>
-    <t>loads_5</t>
-  </si>
-  <si>
     <t>Total number of cycles</t>
   </si>
   <si>
@@ -184,6 +175,24 @@
   </si>
   <si>
     <t>Delta sigma -</t>
+  </si>
+  <si>
+    <t>(loads, 1)</t>
+  </si>
+  <si>
+    <t>(loads, 2)</t>
+  </si>
+  <si>
+    <t>(loads, 3)</t>
+  </si>
+  <si>
+    <t>(loads, 4)</t>
+  </si>
+  <si>
+    <t>loads, 5-1</t>
+  </si>
+  <si>
+    <t>loads, 5-2</t>
   </si>
 </sst>
 </file>
@@ -575,12 +584,15 @@
   <dimension ref="A1:K8"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="11" width="13.69140625" customWidth="1"/>
+    <col min="2" max="7" width="13.69140625" customWidth="1"/>
+    <col min="8" max="8" width="16.23046875" customWidth="1"/>
+    <col min="9" max="9" width="17.23046875" customWidth="1"/>
+    <col min="10" max="11" width="13.69140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="29.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="9" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -636,10 +648,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>13</v>
+        <v>49</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>13</v>
+        <v>49</v>
       </c>
       <c r="J2" s="6" t="s">
         <v>14</v>
@@ -671,10 +683,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>18</v>
+        <v>50</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>18</v>
+        <v>50</v>
       </c>
       <c r="J3" s="4" t="s">
         <v>19</v>
@@ -706,16 +718,16 @@
         <v>0</v>
       </c>
       <c r="H4" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J4" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="I4" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="J4" s="4" t="s">
+      <c r="K4" s="4" t="s">
         <v>23</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.4">
@@ -723,13 +735,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>11</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>12</v>
@@ -741,16 +753,16 @@
         <v>0</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>13</v>
+        <v>49</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>13</v>
+        <v>49</v>
       </c>
       <c r="J5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K5" s="4" t="s">
         <v>23</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.4">
@@ -758,13 +770,13 @@
         <v>1</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>11</v>
       </c>
       <c r="D6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>12</v>
@@ -776,16 +788,16 @@
         <v>0</v>
       </c>
       <c r="H6" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="K6" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.4">
@@ -793,7 +805,7 @@
         <v>1</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>11</v>
@@ -802,7 +814,7 @@
         <v>21</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F7" s="5">
         <v>300</v>
@@ -811,16 +823,16 @@
         <v>0</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.4">
@@ -828,10 +840,10 @@
         <v>1</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D8" t="s">
         <v>12</v>
@@ -846,10 +858,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="J8" s="6" t="s">
         <v>14</v>
@@ -873,7 +885,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="29.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="10" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -894,16 +906,16 @@
         <v>5</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="L1" s="2" t="s">
         <v>8</v>
@@ -970,16 +982,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.4">
@@ -987,10 +999,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D2" s="7">
         <v>1000000</v>
@@ -1001,10 +1013,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D3" s="7">
         <v>1000000</v>
@@ -1026,18 +1038,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A1" s="8" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove the creation of excel files
</commit_message>
<xml_diff>
--- a/tests/bolts/res/Flange1.xlsx
+++ b/tests/bolts/res/Flange1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATA\laghida\Documents\GitLab\cassy\tests\bolts\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DF3670D-C405-47F8-832A-B70F76F4E489}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D041626-9011-4063-9C77-6D6FF01A8BC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="REs" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="56">
   <si>
     <t>ID</t>
   </si>
@@ -193,6 +193,9 @@
   </si>
   <si>
     <t>loads, 5-2</t>
+  </si>
+  <si>
+    <t>loads_3</t>
   </si>
 </sst>
 </file>
@@ -582,15 +585,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K8"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="7" width="13.69140625" customWidth="1"/>
-    <col min="8" max="8" width="16.23046875" customWidth="1"/>
-    <col min="9" max="9" width="17.23046875" customWidth="1"/>
-    <col min="10" max="11" width="13.69140625" customWidth="1"/>
+    <col min="2" max="7" width="13.6640625" customWidth="1"/>
+    <col min="8" max="8" width="16.21875" customWidth="1"/>
+    <col min="9" max="9" width="17.21875" customWidth="1"/>
+    <col min="10" max="11" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="29.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="9" t="s">
         <v>36</v>
       </c>
@@ -625,7 +628,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -660,7 +663,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -695,7 +698,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1</v>
       </c>
@@ -730,7 +733,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1</v>
       </c>
@@ -765,7 +768,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>1</v>
       </c>
@@ -800,7 +803,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1</v>
       </c>
@@ -835,7 +838,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>1</v>
       </c>
@@ -877,13 +880,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED687A43-EC33-423B-A6DD-5E62238FF478}">
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:M3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="13" width="15.69140625" customWidth="1"/>
+    <col min="2" max="13" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="29.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:13" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>36</v>
       </c>
@@ -924,7 +927,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -962,6 +965,47 @@
         <v>14</v>
       </c>
       <c r="M2" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3">
+        <v>100</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3" s="7">
+        <v>10000</v>
+      </c>
+      <c r="I3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J3" t="s">
+        <v>55</v>
+      </c>
+      <c r="K3" t="s">
+        <v>13</v>
+      </c>
+      <c r="L3" t="s">
+        <v>14</v>
+      </c>
+      <c r="M3" t="s">
         <v>15</v>
       </c>
     </row>
@@ -973,14 +1017,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE19EBD1-4CCE-4BC0-AB0E-DF85D1968C61}">
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="11.921875" customWidth="1"/>
-    <col min="3" max="3" width="10.3046875" customWidth="1"/>
+    <col min="2" max="2" width="11.88671875" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>36</v>
       </c>
@@ -994,7 +1038,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1008,7 +1052,7 @@
         <v>1000000</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1030,13 +1074,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{104CCDBF-B7FA-4C2C-914E-1618DEA9FA0D}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.921875" customWidth="1"/>
+    <col min="1" max="1" width="11.88671875" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>45</v>
       </c>
@@ -1044,7 +1088,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>43</v>
       </c>

</xml_diff>

<commit_message>
add windows tag for runner
</commit_message>
<xml_diff>
--- a/tests/bolts/res/Flange1.xlsx
+++ b/tests/bolts/res/Flange1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATA\laghida\Documents\GitLab\cassy\tests\bolts\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DF3670D-C405-47F8-832A-B70F76F4E489}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D041626-9011-4063-9C77-6D6FF01A8BC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="REs" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="56">
   <si>
     <t>ID</t>
   </si>
@@ -193,6 +193,9 @@
   </si>
   <si>
     <t>loads, 5-2</t>
+  </si>
+  <si>
+    <t>loads_3</t>
   </si>
 </sst>
 </file>
@@ -582,15 +585,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K8"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="7" width="13.69140625" customWidth="1"/>
-    <col min="8" max="8" width="16.23046875" customWidth="1"/>
-    <col min="9" max="9" width="17.23046875" customWidth="1"/>
-    <col min="10" max="11" width="13.69140625" customWidth="1"/>
+    <col min="2" max="7" width="13.6640625" customWidth="1"/>
+    <col min="8" max="8" width="16.21875" customWidth="1"/>
+    <col min="9" max="9" width="17.21875" customWidth="1"/>
+    <col min="10" max="11" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="29.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="9" t="s">
         <v>36</v>
       </c>
@@ -625,7 +628,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -660,7 +663,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -695,7 +698,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1</v>
       </c>
@@ -730,7 +733,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1</v>
       </c>
@@ -765,7 +768,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>1</v>
       </c>
@@ -800,7 +803,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1</v>
       </c>
@@ -835,7 +838,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>1</v>
       </c>
@@ -877,13 +880,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED687A43-EC33-423B-A6DD-5E62238FF478}">
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:M3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="13" width="15.69140625" customWidth="1"/>
+    <col min="2" max="13" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="29.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:13" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>36</v>
       </c>
@@ -924,7 +927,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -962,6 +965,47 @@
         <v>14</v>
       </c>
       <c r="M2" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3">
+        <v>100</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3" s="7">
+        <v>10000</v>
+      </c>
+      <c r="I3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J3" t="s">
+        <v>55</v>
+      </c>
+      <c r="K3" t="s">
+        <v>13</v>
+      </c>
+      <c r="L3" t="s">
+        <v>14</v>
+      </c>
+      <c r="M3" t="s">
         <v>15</v>
       </c>
     </row>
@@ -973,14 +1017,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE19EBD1-4CCE-4BC0-AB0E-DF85D1968C61}">
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="11.921875" customWidth="1"/>
-    <col min="3" max="3" width="10.3046875" customWidth="1"/>
+    <col min="2" max="2" width="11.88671875" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>36</v>
       </c>
@@ -994,7 +1038,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1008,7 +1052,7 @@
         <v>1000000</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1030,13 +1074,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{104CCDBF-B7FA-4C2C-914E-1618DEA9FA0D}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.921875" customWidth="1"/>
+    <col min="1" max="1" width="11.88671875" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>45</v>
       </c>
@@ -1044,7 +1088,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>43</v>
       </c>

</xml_diff>